<commit_message>
Added skill standards to questions
</commit_message>
<xml_diff>
--- a/Global/April CMA/Global April CMA Data.xlsx
+++ b/Global/April CMA/Global April CMA Data.xlsx
@@ -40085,7 +40085,11 @@
           <t>8. Effect</t>
         </is>
       </c>
-      <c r="L2" s="25" t="n"/>
+      <c r="L2" s="25" t="inlineStr">
+        <is>
+          <t>B. Chronological Reasoning and Causation</t>
+        </is>
+      </c>
       <c r="M2" s="25" t="inlineStr">
         <is>
           <t>10.01b.1</t>
@@ -40169,7 +40173,11 @@
           <t>14. Stakeholder</t>
         </is>
       </c>
-      <c r="L3" s="25" t="n"/>
+      <c r="L3" s="25" t="inlineStr">
+        <is>
+          <t>C. Comparison and Contextualization</t>
+        </is>
+      </c>
       <c r="M3" s="25" t="inlineStr">
         <is>
           <t>10.02c.1</t>
@@ -40253,7 +40261,11 @@
           <t>4. Claim Validity (Without Outside Information)</t>
         </is>
       </c>
-      <c r="L4" s="25" t="n"/>
+      <c r="L4" s="25" t="inlineStr">
+        <is>
+          <t>A. Gathering, Interpreting, and Using Evidence</t>
+        </is>
+      </c>
       <c r="M4" s="25" t="inlineStr">
         <is>
           <t>10.02c.1</t>
@@ -40337,7 +40349,11 @@
           <t>7. Cause</t>
         </is>
       </c>
-      <c r="L5" s="25" t="n"/>
+      <c r="L5" s="25" t="inlineStr">
+        <is>
+          <t>B. Chronological Reasoning and Causation</t>
+        </is>
+      </c>
       <c r="M5" s="25" t="inlineStr">
         <is>
           <t>10.03b.1</t>
@@ -40421,7 +40437,11 @@
           <t>7. Cause</t>
         </is>
       </c>
-      <c r="L6" s="25" t="n"/>
+      <c r="L6" s="25" t="inlineStr">
+        <is>
+          <t>B. Chronological Reasoning and Causation</t>
+        </is>
+      </c>
       <c r="M6" s="25" t="inlineStr">
         <is>
           <t>10.03c.1</t>
@@ -40505,7 +40525,11 @@
           <t>8. Effect</t>
         </is>
       </c>
-      <c r="L7" s="25" t="n"/>
+      <c r="L7" s="25" t="inlineStr">
+        <is>
+          <t>B. Chronological Reasoning and Causation</t>
+        </is>
+      </c>
       <c r="M7" s="25" t="inlineStr">
         <is>
           <t>10.05a.1</t>
@@ -40589,7 +40613,11 @@
           <t>2. POV</t>
         </is>
       </c>
-      <c r="L8" s="25" t="n"/>
+      <c r="L8" s="25" t="inlineStr">
+        <is>
+          <t>A. Gathering, Interpreting, and Using Evidence</t>
+        </is>
+      </c>
       <c r="M8" s="25" t="inlineStr">
         <is>
           <t>10.05a.1</t>
@@ -40673,7 +40701,11 @@
           <t>1. Best Use</t>
         </is>
       </c>
-      <c r="L9" s="25" t="n"/>
+      <c r="L9" s="25" t="inlineStr">
+        <is>
+          <t>A. Gathering, Interpreting, and Using Evidence</t>
+        </is>
+      </c>
       <c r="M9" s="25" t="inlineStr">
         <is>
           <t>10.05b.1</t>
@@ -40757,7 +40789,11 @@
           <t>4. Claim Validity (Without Outside Information)</t>
         </is>
       </c>
-      <c r="L10" s="25" t="n"/>
+      <c r="L10" s="25" t="inlineStr">
+        <is>
+          <t>A. Gathering, Interpreting, and Using Evidence</t>
+        </is>
+      </c>
       <c r="M10" s="25" t="inlineStr">
         <is>
           <t>10.05b.1</t>
@@ -40841,7 +40877,11 @@
           <t>7. Cause</t>
         </is>
       </c>
-      <c r="L11" s="25" t="n"/>
+      <c r="L11" s="25" t="inlineStr">
+        <is>
+          <t>B. Chronological Reasoning and Causation</t>
+        </is>
+      </c>
       <c r="M11" s="25" t="inlineStr">
         <is>
           <t>10.05d.4</t>
@@ -40925,7 +40965,11 @@
           <t>10. Similarity</t>
         </is>
       </c>
-      <c r="L12" s="25" t="n"/>
+      <c r="L12" s="25" t="inlineStr">
+        <is>
+          <t>C. Comparison and Contextualization</t>
+        </is>
+      </c>
       <c r="M12" s="25" t="inlineStr">
         <is>
           <t>10.05d.4</t>
@@ -41009,7 +41053,11 @@
           <t>7. Cause</t>
         </is>
       </c>
-      <c r="L13" s="25" t="n"/>
+      <c r="L13" s="25" t="inlineStr">
+        <is>
+          <t>B. Chronological Reasoning and Causation</t>
+        </is>
+      </c>
       <c r="M13" s="25" t="inlineStr">
         <is>
           <t>10.05d.2</t>
@@ -41093,7 +41141,11 @@
           <t>4. Claim Validity (Without Outside Information)</t>
         </is>
       </c>
-      <c r="L14" s="25" t="n"/>
+      <c r="L14" s="25" t="inlineStr">
+        <is>
+          <t>B. Chronological Reasoning and Causation</t>
+        </is>
+      </c>
       <c r="M14" s="25" t="inlineStr">
         <is>
           <t>10.05d.2</t>
@@ -41177,7 +41229,11 @@
           <t>1. Best Use</t>
         </is>
       </c>
-      <c r="L15" s="25" t="n"/>
+      <c r="L15" s="25" t="inlineStr">
+        <is>
+          <t>A. Gathering, Interpreting, and Using Evidence</t>
+        </is>
+      </c>
       <c r="M15" s="25" t="inlineStr">
         <is>
           <t>10.05b.1</t>
@@ -41261,7 +41317,11 @@
           <t>8. Effect</t>
         </is>
       </c>
-      <c r="L16" s="25" t="n"/>
+      <c r="L16" s="25" t="inlineStr">
+        <is>
+          <t>B. Chronological Reasoning and Causation</t>
+        </is>
+      </c>
       <c r="M16" s="25" t="inlineStr">
         <is>
           <t>10.05b.1</t>
@@ -41345,7 +41405,11 @@
           <t>6. Significance of Event/Development</t>
         </is>
       </c>
-      <c r="L17" s="25" t="n"/>
+      <c r="L17" s="25" t="inlineStr">
+        <is>
+          <t>C. Comparison and Contextualization</t>
+        </is>
+      </c>
       <c r="M17" s="25" t="inlineStr">
         <is>
           <t>10.06a.1</t>
@@ -41429,7 +41493,11 @@
           <t>15. Course of Action</t>
         </is>
       </c>
-      <c r="L18" s="25" t="n"/>
+      <c r="L18" s="25" t="inlineStr">
+        <is>
+          <t>A. Gathering, Interpreting, and Using Evidence</t>
+        </is>
+      </c>
       <c r="M18" s="25" t="inlineStr">
         <is>
           <t>10.06a.1</t>

</xml_diff>